<commit_message>
Benhcmark results PC - 11.07
</commit_message>
<xml_diff>
--- a/analysis/results/PC/comparison.xlsx
+++ b/analysis/results/PC/comparison.xlsx
@@ -561,13 +561,13 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.5611</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.5588</v>
+        <v>0.5637</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.5595</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0.0337</v>
@@ -593,13 +593,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.8398</v>
+        <v>1.803</v>
       </c>
       <c r="D3" t="n">
-        <v>1.7482</v>
+        <v>1.7319</v>
       </c>
       <c r="E3" t="n">
-        <v>2.2714</v>
+        <v>2.1115</v>
       </c>
       <c r="F3" t="n">
         <v>0.0387</v>
@@ -637,13 +637,13 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.8369</v>
+        <v>1.8191</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1.7582</v>
+        <v>1.7372</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1.9731</v>
+        <v>1.882</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>0.0394</v>
@@ -679,19 +679,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.9653</v>
+        <v>1.9641</v>
       </c>
       <c r="D5" t="n">
-        <v>1.8131</v>
+        <v>1.9051</v>
       </c>
       <c r="E5" t="n">
-        <v>2.0835</v>
+        <v>2.0346</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0723</v>
+        <v>0.0698</v>
       </c>
       <c r="G5" t="n">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -721,16 +721,16 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4.0883</v>
+        <v>4.0597</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>4.0163</v>
+        <v>3.9708</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>4.6358</v>
+        <v>4.3134</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.5049</v>
+        <v>0.5219</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>4608</v>
@@ -763,16 +763,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>24.5687</v>
+        <v>24.5602</v>
       </c>
       <c r="D7" t="n">
-        <v>24.2407</v>
+        <v>24.3312</v>
       </c>
       <c r="E7" t="n">
-        <v>25.5795</v>
+        <v>25.325</v>
       </c>
       <c r="F7" t="n">
-        <v>6.2018</v>
+        <v>6.2968</v>
       </c>
       <c r="G7" t="n">
         <v>41229</v>
@@ -805,16 +805,16 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>227.233</v>
+        <v>228.0876</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>225.4904</v>
+        <v>226.341</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>230.9373</v>
+        <v>238.8597</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>63.7461</v>
+        <v>63.3234</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>407490</v>
@@ -847,16 +847,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>79.81570000000001</v>
+        <v>1.0677</v>
       </c>
       <c r="D9" t="n">
-        <v>79.0234</v>
+        <v>1.245</v>
       </c>
       <c r="E9" t="n">
-        <v>80.49339999999999</v>
+        <v>1.0394</v>
       </c>
       <c r="F9" t="n">
-        <v>135.1825</v>
+        <v>0.0138</v>
       </c>
       <c r="G9" t="n">
         <v>291</v>
@@ -891,16 +891,16 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>79.7383</v>
+        <v>1.0718</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>78.8899</v>
+        <v>1.3537</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>80.6165</v>
+        <v>1.0921</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>135.2485</v>
+        <v>0.014</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>470</v>
@@ -933,19 +933,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>79.84059999999999</v>
+        <v>1.1264</v>
       </c>
       <c r="D11" t="n">
-        <v>78.8198</v>
+        <v>1.4341</v>
       </c>
       <c r="E11" t="n">
-        <v>80.1626</v>
+        <v>1.1288</v>
       </c>
       <c r="F11" t="n">
-        <v>135.1993</v>
+        <v>0.05</v>
       </c>
       <c r="G11" t="n">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -975,16 +975,16 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>79.8235</v>
+        <v>1.3612</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>79.4182</v>
+        <v>1.794</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>80.98569999999999</v>
+        <v>1.388</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>135.3995</v>
+        <v>0.4085</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>4608</v>
@@ -1017,16 +1017,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>82.55029999999999</v>
+        <v>3.6635</v>
       </c>
       <c r="D13" t="n">
-        <v>81.604</v>
+        <v>4.1346</v>
       </c>
       <c r="E13" t="n">
-        <v>83.08839999999999</v>
+        <v>3.7495</v>
       </c>
       <c r="F13" t="n">
-        <v>139.529</v>
+        <v>3.7165</v>
       </c>
       <c r="G13" t="n">
         <v>41229</v>
@@ -1059,16 +1059,16 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>110.6476</v>
+        <v>32.7058</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>109.8422</v>
+        <v>32.7759</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>111.5141</v>
+        <v>32.187</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>178.5258</v>
+        <v>43.4796</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>407490</v>
@@ -1106,7 +1106,7 @@
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -1215,13 +1215,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.5611</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5588</v>
+        <v>0.5637</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5595</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="F2" t="n">
         <v>20</v>
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>78.03870000000001</v>
+        <v>78.0018</v>
       </c>
       <c r="D3" t="n">
-        <v>78.0027</v>
+        <v>77.98309999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>78.9986</v>
+        <v>78.0592</v>
       </c>
       <c r="F3" t="n">
         <v>20</v>
@@ -1339,13 +1339,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.8398</v>
+        <v>1.803</v>
       </c>
       <c r="D4" t="n">
-        <v>1.7482</v>
+        <v>1.7319</v>
       </c>
       <c r="E4" t="n">
-        <v>2.2714</v>
+        <v>2.1115</v>
       </c>
       <c r="F4" t="n">
         <v>20</v>
@@ -1401,13 +1401,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.8369</v>
+        <v>1.8191</v>
       </c>
       <c r="D5" t="n">
-        <v>1.7582</v>
+        <v>1.7372</v>
       </c>
       <c r="E5" t="n">
-        <v>1.9731</v>
+        <v>1.882</v>
       </c>
       <c r="F5" t="n">
         <v>20</v>
@@ -1463,13 +1463,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.9653</v>
+        <v>1.9641</v>
       </c>
       <c r="D6" t="n">
-        <v>1.8131</v>
+        <v>1.9051</v>
       </c>
       <c r="E6" t="n">
-        <v>2.0835</v>
+        <v>2.0346</v>
       </c>
       <c r="F6" t="n">
         <v>20</v>
@@ -1478,7 +1478,7 @@
         <v>65536</v>
       </c>
       <c r="H6" t="n">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1525,13 +1525,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4.0883</v>
+        <v>4.0597</v>
       </c>
       <c r="D7" t="n">
-        <v>4.0163</v>
+        <v>3.9708</v>
       </c>
       <c r="E7" t="n">
-        <v>4.6358</v>
+        <v>4.3134</v>
       </c>
       <c r="F7" t="n">
         <v>20</v>
@@ -1587,13 +1587,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24.5687</v>
+        <v>24.5602</v>
       </c>
       <c r="D8" t="n">
-        <v>24.2407</v>
+        <v>24.3312</v>
       </c>
       <c r="E8" t="n">
-        <v>25.5795</v>
+        <v>25.325</v>
       </c>
       <c r="F8" t="n">
         <v>20</v>
@@ -1649,13 +1649,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>227.233</v>
+        <v>228.0876</v>
       </c>
       <c r="D9" t="n">
-        <v>225.4904</v>
+        <v>226.341</v>
       </c>
       <c r="E9" t="n">
-        <v>230.9373</v>
+        <v>238.8597</v>
       </c>
       <c r="F9" t="n">
         <v>20</v>
@@ -1711,13 +1711,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>79.81570000000001</v>
+        <v>1.0677</v>
       </c>
       <c r="D10" t="n">
-        <v>79.0234</v>
+        <v>1.245</v>
       </c>
       <c r="E10" t="n">
-        <v>80.49339999999999</v>
+        <v>1.0394</v>
       </c>
       <c r="F10" t="n">
         <v>20</v>
@@ -1773,13 +1773,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>79.7383</v>
+        <v>1.0718</v>
       </c>
       <c r="D11" t="n">
-        <v>78.8899</v>
+        <v>1.3537</v>
       </c>
       <c r="E11" t="n">
-        <v>80.6165</v>
+        <v>1.0921</v>
       </c>
       <c r="F11" t="n">
         <v>20</v>
@@ -1835,13 +1835,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>79.84059999999999</v>
+        <v>1.1264</v>
       </c>
       <c r="D12" t="n">
-        <v>78.8198</v>
+        <v>1.4341</v>
       </c>
       <c r="E12" t="n">
-        <v>80.1626</v>
+        <v>1.1288</v>
       </c>
       <c r="F12" t="n">
         <v>20</v>
@@ -1897,13 +1897,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>79.8235</v>
+        <v>1.3612</v>
       </c>
       <c r="D13" t="n">
-        <v>79.4182</v>
+        <v>1.794</v>
       </c>
       <c r="E13" t="n">
-        <v>80.98569999999999</v>
+        <v>1.388</v>
       </c>
       <c r="F13" t="n">
         <v>20</v>
@@ -1959,13 +1959,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>82.55029999999999</v>
+        <v>3.6635</v>
       </c>
       <c r="D14" t="n">
-        <v>81.604</v>
+        <v>4.1346</v>
       </c>
       <c r="E14" t="n">
-        <v>83.08839999999999</v>
+        <v>3.7495</v>
       </c>
       <c r="F14" t="n">
         <v>20</v>
@@ -2021,13 +2021,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>110.6476</v>
+        <v>32.7058</v>
       </c>
       <c r="D15" t="n">
-        <v>109.8422</v>
+        <v>32.7759</v>
       </c>
       <c r="E15" t="n">
-        <v>111.5141</v>
+        <v>32.187</v>
       </c>
       <c r="F15" t="n">
         <v>20</v>
@@ -2222,7 +2222,7 @@
         <v>65536</v>
       </c>
       <c r="H18" t="n">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
@@ -2284,7 +2284,7 @@
         <v>1048576</v>
       </c>
       <c r="H19" t="n">
-        <v>4611</v>
+        <v>4612</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
@@ -2459,9 +2459,9 @@
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -2545,16 +2545,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.0337</v>
+        <v>0.033736</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0337</v>
+        <v>0.033736</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0337</v>
+        <v>0.033736</v>
       </c>
       <c r="F2" t="n">
-        <v>353353</v>
+        <v>356763</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -2595,13 +2595,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>78.33337</v>
+        <v>78.407263</v>
       </c>
       <c r="D3" t="n">
-        <v>78.33337</v>
+        <v>78.407263</v>
       </c>
       <c r="E3" t="n">
-        <v>78.33337</v>
+        <v>78.407263</v>
       </c>
       <c r="F3" t="n">
         <v>152</v>
@@ -2645,16 +2645,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.038748</v>
+        <v>0.038697</v>
       </c>
       <c r="D4" t="n">
-        <v>0.038748</v>
+        <v>0.038697</v>
       </c>
       <c r="E4" t="n">
-        <v>0.038748</v>
+        <v>0.038697</v>
       </c>
       <c r="F4" t="n">
-        <v>310849</v>
+        <v>308029</v>
       </c>
       <c r="G4" t="n">
         <v>100</v>
@@ -2695,16 +2695,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.039427</v>
+        <v>0.039406</v>
       </c>
       <c r="D5" t="n">
-        <v>0.039427</v>
+        <v>0.039406</v>
       </c>
       <c r="E5" t="n">
-        <v>0.039427</v>
+        <v>0.039406</v>
       </c>
       <c r="F5" t="n">
-        <v>302682</v>
+        <v>303489</v>
       </c>
       <c r="G5" t="n">
         <v>1024</v>
@@ -2745,16 +2745,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.072296</v>
+        <v>0.06983200000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>0.072296</v>
+        <v>0.06983200000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>0.072296</v>
+        <v>0.06983200000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>167623</v>
+        <v>166675</v>
       </c>
       <c r="G6" t="n">
         <v>65536</v>
@@ -2795,16 +2795,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.504906</v>
+        <v>0.521865</v>
       </c>
       <c r="D7" t="n">
-        <v>0.504906</v>
+        <v>0.521865</v>
       </c>
       <c r="E7" t="n">
-        <v>0.504906</v>
+        <v>0.521865</v>
       </c>
       <c r="F7" t="n">
-        <v>25104</v>
+        <v>25056</v>
       </c>
       <c r="G7" t="n">
         <v>1048576</v>
@@ -2845,16 +2845,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.201794</v>
+        <v>6.296836</v>
       </c>
       <c r="D8" t="n">
-        <v>6.201794</v>
+        <v>6.296836</v>
       </c>
       <c r="E8" t="n">
-        <v>6.201794</v>
+        <v>6.296836</v>
       </c>
       <c r="F8" t="n">
-        <v>1890</v>
+        <v>1869</v>
       </c>
       <c r="G8" t="n">
         <v>10485760</v>
@@ -2895,16 +2895,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>63.746074</v>
+        <v>63.323358</v>
       </c>
       <c r="D9" t="n">
-        <v>63.746074</v>
+        <v>63.323358</v>
       </c>
       <c r="E9" t="n">
-        <v>63.746074</v>
+        <v>63.323358</v>
       </c>
       <c r="F9" t="n">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G9" t="n">
         <v>104857600</v>
@@ -2945,16 +2945,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>135.182467</v>
+        <v>0.013816</v>
       </c>
       <c r="D10" t="n">
-        <v>135.182467</v>
+        <v>0.013816</v>
       </c>
       <c r="E10" t="n">
-        <v>135.182467</v>
+        <v>0.013816</v>
       </c>
       <c r="F10" t="n">
-        <v>88</v>
+        <v>883281</v>
       </c>
       <c r="G10" t="n">
         <v>100</v>
@@ -2995,16 +2995,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>135.248458</v>
+        <v>0.013971</v>
       </c>
       <c r="D11" t="n">
-        <v>135.248458</v>
+        <v>0.013971</v>
       </c>
       <c r="E11" t="n">
-        <v>135.248458</v>
+        <v>0.013971</v>
       </c>
       <c r="F11" t="n">
-        <v>88</v>
+        <v>862858</v>
       </c>
       <c r="G11" t="n">
         <v>1024</v>
@@ -3045,16 +3045,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>135.199346</v>
+        <v>0.050022</v>
       </c>
       <c r="D12" t="n">
-        <v>135.199346</v>
+        <v>0.050022</v>
       </c>
       <c r="E12" t="n">
-        <v>135.199346</v>
+        <v>0.050022</v>
       </c>
       <c r="F12" t="n">
-        <v>87</v>
+        <v>236608</v>
       </c>
       <c r="G12" t="n">
         <v>65536</v>
@@ -3095,16 +3095,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>135.399485</v>
+        <v>0.408488</v>
       </c>
       <c r="D13" t="n">
-        <v>135.399485</v>
+        <v>0.408488</v>
       </c>
       <c r="E13" t="n">
-        <v>135.399485</v>
+        <v>0.408488</v>
       </c>
       <c r="F13" t="n">
-        <v>88</v>
+        <v>29388</v>
       </c>
       <c r="G13" t="n">
         <v>1048576</v>
@@ -3145,16 +3145,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>139.528984</v>
+        <v>3.716526</v>
       </c>
       <c r="D14" t="n">
-        <v>139.528984</v>
+        <v>3.716526</v>
       </c>
       <c r="E14" t="n">
-        <v>139.528984</v>
+        <v>3.716526</v>
       </c>
       <c r="F14" t="n">
-        <v>85</v>
+        <v>3195</v>
       </c>
       <c r="G14" t="n">
         <v>10485760</v>
@@ -3195,16 +3195,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>178.525776</v>
+        <v>43.479608</v>
       </c>
       <c r="D15" t="n">
-        <v>178.525776</v>
+        <v>43.479608</v>
       </c>
       <c r="E15" t="n">
-        <v>178.525776</v>
+        <v>43.479608</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>276</v>
       </c>
       <c r="G15" t="n">
         <v>104857600</v>

</xml_diff>